<commit_message>
perbaiki berbagai masalah import data SBM(nanti di test lagi)
</commit_message>
<xml_diff>
--- a/backend/storage/imports/Master_SBM/1. SATUAN BIAYA TRANSPORTASI DARAT DARI IBUKOTA PROVINSI KE KABUPATEN atau KOTA DALAM PROVINSI YANG SAMA (ONE  WAY ).xlsx
+++ b/backend/storage/imports/Master_SBM/1. SATUAN BIAYA TRANSPORTASI DARAT DARI IBUKOTA PROVINSI KE KABUPATEN atau KOTA DALAM PROVINSI YANG SAMA (ONE  WAY ).xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\dokumen perkuliahan\kebutuhan magang\Projek magang\DITUGASKAN\SBM\baru\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\dokumen perkuliahan\kebutuhan magang\Projek magang\DITUGASKAN\SBM\baru 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDC82306-88BB-4766-A3F6-EAACB0FEF6AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB442C87-250E-487D-BA7C-65B9D30ED8F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5B7BDC6F-2136-4638-AE5D-449A58C3D81C}"/>
   </bookViews>

</xml_diff>